<commit_message>
Updated Case Study 2025
</commit_message>
<xml_diff>
--- a/Codes_2025/Trial 3/Trial3_ARIMAX_Followers_Results.xlsx
+++ b/Codes_2025/Trial 3/Trial3_ARIMAX_Followers_Results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,17 +609,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>37.81</v>
+        <v>19.89</v>
       </c>
       <c r="D6" t="n">
-        <v>37.78722367369897</v>
+        <v>16.07043810532318</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -628,11 +628,11 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>(2,1,1)</t>
+          <t>(2,1,0)</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.02277632630102744</v>
+        <v>3.819561894676816</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -643,17 +643,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>6.81</v>
+        <v>8.050000000000002</v>
       </c>
       <c r="D7" t="n">
-        <v>10.71819864477671</v>
+        <v>20.0793601323844</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -662,11 +662,11 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>(0,1,0)</t>
+          <t>(2,1,0)</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>3.908198644776713</v>
+        <v>12.0293601323844</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -677,17 +677,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>2025</v>
       </c>
       <c r="C8" t="n">
-        <v>19.89</v>
+        <v>7.989999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>16.07043810532318</v>
+        <v>13.45660008868974</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -696,11 +696,11 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>(2,1,0)</t>
+          <t>(0,1,0)</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>3.819561894676816</v>
+        <v>5.466600088689737</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -711,17 +711,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>2025</v>
       </c>
       <c r="C9" t="n">
-        <v>8.050000000000002</v>
+        <v>28.09</v>
       </c>
       <c r="D9" t="n">
-        <v>20.0793601323844</v>
+        <v>34.53127418221176</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>12.0293601323844</v>
+        <v>6.441274182211764</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -745,17 +745,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Malta</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>2025</v>
       </c>
       <c r="C10" t="n">
-        <v>7.989999999999999</v>
+        <v>33.88</v>
       </c>
       <c r="D10" t="n">
-        <v>13.45660008868974</v>
+        <v>138.2782907189612</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -764,11 +764,11 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>(0,1,0)</t>
+          <t>(0,1,1)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>5.466600088689737</v>
+        <v>104.3982907189612</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -779,17 +779,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>2025</v>
       </c>
       <c r="C11" t="n">
-        <v>28.09</v>
+        <v>5.56</v>
       </c>
       <c r="D11" t="n">
-        <v>34.53127418221176</v>
+        <v>3.665586312437117</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -798,11 +798,11 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>(2,1,0)</t>
+          <t>(0,1,0)</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>6.441274182211764</v>
+        <v>1.894413687562882</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -813,17 +813,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Malta</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2025</v>
       </c>
       <c r="C12" t="n">
-        <v>33.88</v>
+        <v>11.6</v>
       </c>
       <c r="D12" t="n">
-        <v>138.2782907189612</v>
+        <v>9.046024639142363</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -832,115 +832,13 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>(0,1,1)</t>
+          <t>(2,1,1)</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>104.3982907189612</v>
+        <v>2.553975360857638</v>
       </c>
       <c r="H12" t="inlineStr">
-        <is>
-          <t>Followers</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C13" t="n">
-        <v>24.26000000000001</v>
-      </c>
-      <c r="D13" t="n">
-        <v>37.37242473622501</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>(2,1,1)</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>13.11242473622501</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Followers</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Slovakia</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C14" t="n">
-        <v>5.56</v>
-      </c>
-      <c r="D14" t="n">
-        <v>3.665586312437117</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>(0,1,0)</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>1.894413687562882</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Followers</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Slovenia</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C15" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="D15" t="n">
-        <v>9.046024639142363</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>(2,1,1)</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>2.553975360857638</v>
-      </c>
-      <c r="H15" t="inlineStr">
         <is>
           <t>Followers</t>
         </is>

</xml_diff>